<commit_message>
Fix live-transfer and restore-destination bugs found on the two-machine test
- BUG-024: capture selection field names now match the TS wire format
  (rename_all camelCase + deny_unknown_fields); Policy kept snake_case via
  per-field aliases. New ipc_selection_contract.ts pins the agreement.
- BUG-025: discovered device names strip the mDNS service suffix.
- BUG-026: send resolved destinations from a map nothing ever populated;
  it now reads discovery's map first. resolve_destination extracted + tested.
- BUG-027: a bucket with one project uses the typed folder exactly;
  several projects nest beneath it. No more source-folder-name leakage.
- Trust scope vocabularies unified in @lib/trustScopes (requested vs stored).
  DevicesScreen/TransferScreen use canReceive()/scopeLabel().
- 15 new frontend tests (99 total); 377 Rust tests.
</commit_message>
<xml_diff>
--- a/WorkspaceClone_Tracking.xlsx
+++ b/WorkspaceClone_Tracking.xlsx
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I68"/>
+  <dimension ref="A1:I75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4037,6 +4037,335 @@
       <c r="I68" t="inlineStr">
         <is>
           <t>codesign,tauri-config,root-cause,bug-023</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>LOG-072</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:05</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>BUG</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>IPC / Capture</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>BUG-024</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Live two-machine test: sending a workspace failed on a casing mismatch</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>First real capture-to-send attempt returned `missing field `file_transfer``. Both types were complete and agreed on every name; they disagreed on the convention. Serde ignores unknown keys, so all five misnamed CaptureSelection fields arrived as empty lists, and only the nested Policy's first missing field stopped the command. The error named a field the caller was also sending. Fixed at source on all eleven affected fields across four types, not just the one reported.</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>bug,ipc,capture,serde,live-test</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>LOG-073</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:25</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>IPC / Capture</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Added a cross-language contract test after confirming it fails on the broken code</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>6 tests in adapters/tests/ipc_selection_contract.rs. The central one reads the real src/types/index.ts and compares field names against what serde accepts, placing a gate in the space where the bug lived. Verified by reverting the fix and re-running: 3 tests fail, reproducing the user's exact error. An honest limit was found in the process -- the field-name comparison did not catch removal of the rename_all attribute, because it converts snake_case to camelCase first and so agreed either way. A separate test now pins the convention directly, also confirmed by revert.</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>test,gate,ipc,verification</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>LOG-074</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:10</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Network / Discovery</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>BUG-025</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Device names no longer carry the mDNS service type</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>The laptop was listed as `BISWAJITA._workspace-clone._tcp`. The full name is `{instance}.{service}.{domain}` and only the instance label is a name. Extracted `instance_display_name` to strip the whole service suffix case-insensitively, hoisted SERVICE_TYPE so registration and parsing share one constant, and rewrote the test that had been green while the bug was live. 4 new cases; 5 total. The existing test had asserted no trailing dot and no `.local` and passed happily, checking two properties that held while missing the one that was wrong.</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>bug,discovery,mdns,naming,test</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>LOG-075</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:20</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>DECISION</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Privacy / Browser</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>DEC-029</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Browser history capture is a documented guarantee, not a gap</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>The user reported that open URLs are not shown on the Mac. The browser adapter reports `history_access: "none: URLs are supplied by the user"` and the developer guide promises under 'Never read from your machine at all' that browser tabs, history, profiles and session databases are never read. The capture screen has a 'One URL per line' box. Reading history would retract a documented privacy guarantee on the most sensitive data on a machine, and is not only an adapter change: Chrome's History is SQLite, locked while the browser runs, and gated on macOS behind Full Disk Access. Not implemented. Offered a clipboard-paste shortcut as the honest alternative, which needs no new permission.</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>decision,privacy,browser,scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>LOG-076</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:35</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>TEST</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Network / Transfer</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Added a live probe that tells a bound port from a served one</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>network/examples/live_listener_probe.rs. The receive module's own header records a build where the listener was bound and its port advertised while nothing called accept_once -- the app looked reachable and could receive nothing, and a bound port proves nothing about being served. The probe connects, sends bytes that cannot be a valid Noise handshake, and waits for the app to close: a served loop reads and drops, an unserved one never reads. Validated in both directions -- PASS against the running app, FAIL against a deliberately unserved listener. It cannot prove a transfer succeeds end to end, which needs a paired peer and a workspace.</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>test,network,transfer,verification,tooling</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>LOG-077</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>2026-09-28 20:22</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Network / Transfer</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>BUG-026: send failed on a device discovery could see, because the send path read a map nothing ever populated</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>send_workspace looked up its destination only in TransferService::known, which remember_device() is the only writer of -- and no command ever calls it. known stayed empty for the process's whole life, so every send died with 'No device with id ... is currently reachable' before a socket opened, on a device the UI (reading discovery's own map) showed as on-network, paired and allowed to receive. Fixed by resolving from the discovery service's map first, dropping to known when an mDNS record expires, extracted as pure resolve_destination with 4 new tests; DiscoveryService gained a cfg(test) insert_for_test. Reverted to prove the tests catch the shipped bug (2 fail). 374 Rust tests green.</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>bug,transfer,discovery,resolution,live-test</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>LOG-078</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>2026-09-28 20:40</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Restore / Planner</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>FEAT-040</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>BUG-027: restore nested projects under the destination root, appending the source machine's folder name</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>resolve_destinations resolved root.join(project.name) for every project. The name is the source machine's folder name (openshorts from Documents/openshorts on the Mac), so restoring to E:/workspace-clone produced E:/workspace-clone/openshorts and the report asked the user to create a folder they never named. New rule: one project per bucket lands exactly in the folder typed (name never consulted, hostile names inert); several projects per bucket nest under it via safe_child. Same-name collisions warn. Revert-verified; 377 Rust / 99 vitest green.</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>bug,restore,destination,planner,live-test</t>
         </is>
       </c>
     </row>
@@ -4773,7 +5102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P75"/>
+  <dimension ref="A1:P76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10012,6 +10341,82 @@
       <c r="P75" t="inlineStr">
         <is>
           <t>Done. The mismatch refusal was kept deliberately: the relaxation is 'no number required', not 'no number checked'. The dialog now also tells the user to start a pairing from the other machine, which is what the first live attempt was missing - that was read as a missing feature rather than a two-sided ceremony, so the instruction is now on screen instead of only in the guide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>EPIC-003</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Cross-language field-name contract for IPC payloads</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>A test that reads the real TypeScript interfaces and compares them against the names serde will accept, so a field renamed in either language fails the build instead of silently producing an empty capture.</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>IPC / Capture</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="H76" t="n">
+        <v>100</v>
+      </c>
+      <c r="I76" t="n">
+        <v>1</v>
+      </c>
+      <c r="J76" t="n">
+        <v>1</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="M76" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>BUG-024</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>Renaming or adding a field in either src/types/index.ts or the Rust IPC structs fails the test suite. Verified by reverting the fix and confirming 3 tests fail, reproducing the user's exact error text.</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr">
+        <is>
+          <t>Done. Added in adapters/tests/ipc_selection_contract.rs, 6 tests: the real UI payload deserializes completely; a misspelled key is refused; Policy reads camelCase and still writes snake_case; a manifest round-trips unchanged; the camelCase convention itself is pinned; and TypeScript field names are compared against serde. The gate exists because BUG-024 was invisible to every check in the build. Honest limit recorded in BUG-024: the field-name comparison alone does not catch removal of the rename_all attribute, which is why the convention has its own test. Both confirmed by revert rather than assumed.</t>
         </is>
       </c>
     </row>
@@ -14506,7 +14911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q24"/>
+  <dimension ref="A1:Q28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -16603,6 +17008,354 @@
       <c r="Q24" t="inlineStr">
         <is>
           <t>Was written as 'not yet fixed at source - the DMG predates the fix'. Both statements were superseded within the hour by the signingIdentity change, and the DMG has been rebuilt since. Corrected 2026-09-28. What remains true: this is ad-hoc signing, so a DMG copied to a different Mac is still quarantined by Gatekeeper and needs right-click -&gt; Open. Ad-hoc signing cannot fix that; only notarisation would.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>BUG-024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sending a workspace failed: missing field `file_transfer`</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>The first capture-to-send attempt between the two real machines failed with `invalid args `selection` for command `capture_workspace`: missing field `file_transfer``. The error names a field the UI was in fact sending, so fixing that one field would have produced a second error immediately after.</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>On the Mac, capture a workspace and send it to the paired laptop. The command rejects the payload before the capture begins.</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>The selection deserializes and the workspace transfers.</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>The command was rejected before the capture began, with a message naming `file_transfer` -- a field the UI was sending, under the name it was also sending. Every misnamed list field would have arrived empty, so a capture that got past this would have silently dropped selected projects and pasted URLs while still reporting success; the URLs vanishing would have pointed at the browser adapter, four functions from the actual cause.</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>The capture never started. Rust read the selection as snake_case (`include_applications`, `browser_urls`, `source_path`) and the UI wrote it as camelCase (`includeApplications`, `browserUrls`, `sourcePath`). `CaptureSelection` in adapters/src/traits.rs was the one IPC-boundary type missing `#[serde(rename_all = "camelCase")]`; that convention is applied in 9 other places, all in commands/src/. Because serde ignores unknown keys, all five misnamed fields arrived as empty lists rather than errors, and only the nested `Policy` failing on the first missing field in its declaration order stopped the command -- so the error named a field the caller was also sending.</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Added `#[serde(rename_all = "camelCase", deny_unknown_fields)]` to `CaptureSelection`, `SelectedProject` and `ApprovedCommand` -- all eleven affected fields across all four types, not only the one reported. `Policy` took per-field `alias`es instead (DEC-029), because it is also the manifest's policy: a blanket rename would have fixed the input and silently rewritten the manifest wire format. `deny_unknown_fields` closes the worse half of the bug (DEC-030).</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Yes, at source. Confirmed by reverting the fix and re-running the new contract test: 3 of 6 tests fail, reproducing the user's exact error text, `missing field `file_transfer``.</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:40</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>Three gates were green while this was live: tsc checks TypeScript against its own types, cargo test builds the struct in Rust where naming is irrelevant, and check_command_parity.py compares command *names*. The bug lived in the space between them, so FEAT-075 puts a gate there. Honest limit found while testing the new gate: the field-name comparison alone did NOT catch removal of the rename_all attribute, because it converts snake_case to camelCase first and so agreed either way. A separate test pins the convention directly. Both were confirmed by revert, not assumed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>BUG-025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Discovered devices listed with the mDNS service type glued to the name</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>The paired laptop appeared in the device list as `BISWAJITA._workspace-clone._tcp` rather than `BISWAJITA`.</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>Pair a device and open the Devices screen.</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>The device is listed under the name its owner chose.</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>The name carried `._workspace-clone._tcp`.</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>`parse_discovered_device` took the mDNS full name and stripped the trailing dot and the `.local` domain, but never the service type. The comment beside that code said the goal was a name that helps a person recognise their own machine -- so the code was the bug the comment was warning about, not the one it described.</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Extracted `instance_display_name`, which strips the whole service suffix (case-insensitively, since mDNS names are) rather than a `.local` substring, and hoisted the service type to a `SERVICE_TYPE` constant used by both registration and parsing so the two halves cannot drift. Substring stripping was avoided deliberately: a Mac genuinely named `ABHISHEKs-MacBook-Air.local` must keep its `.local`, or the app would rename a device to something its owner never chose.</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Yes, and the test that was green while the bug was live was the tell.</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:10</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>`the_display_name_is_not_a_dns_name` already existed, asserted that the name has no trailing dot and no `.local`, and passed throughout. It checked two properties that happened to hold while missing the one that was wrong. It now asserts the exact expected value, plus four new cases: a display name that itself ends in `.local`, mixed-case service types, an unrecognised full name, and a degenerate one that must not reduce to empty. The last two guard the 'never lose a device to a naming quirk' rule. Confirmed the strengthened test fails on the old code.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>BUG-026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>FEAT-075</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Send failed: 'No device with id ... is currently reachable' for a device the UI showed as on-network, paired and allowed to receive</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>The first real send attempt on the Mac against the paired laptop failed before a socket was ever opened, with: Network error: Connection failed: No device with id 'hnODGDVs/oYDiOhuQO941A==' is currently reachable. Check that it is running, on the same network, and that discovery has found it on this screen. The device the message denied seeing was simultaneously listed on the very screen the user was looking at, shown as on-network, paired, and permitted to receive.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>On the Mac, with the laptop discovered (the Send button enabled), click Send workspace.</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>The send starts and the transfer proceeds.</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>The send failed with 'No device with id ... is currently reachable' -- the wording telling the user discovery had not found the device, when the screen it told them to check was proving the opposite.</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>send_workspace resolved its destination only from TransferService::known, a second map fed exclusively by remember_device() -- a method nothing in the workspace ever calls, let alone a command. known was therefore empty for the whole lifetime of the process, so every send failed here regardless of what discovery knew. Discovery's own map, the one get_discovered_devices reads and the mDNS browse loop actually fills, was never consulted. The comment above the lookup even claimed peers are found 'in two places ... what discovery has seen on the network right now, and what a previous command recorded' -- only one lookup existed and it read the wrong map. The e2e integration test stayed green because it hands a hand-built peer record straight to TransferService::send_workspace and never exercises the command's destination resolution.</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Resolve the destination from the discovery service's map first (the map the browse loop writes and get_discovered_devices reads), with TransferService::known as the fallback for a record whose mDNS entry has expired. Extracted as a pure function resolve_destination(from_discovery, remembered, device_id) per DEC-026 so the two-source rule is testable; the payload/authorization steps are unchanged and happen before the transfer lock, and the discovery lookup happens before the transfer lock so the two locks are never nested. The error message now distinguishes being unreachable from being untrusted, and no longer tells the user to verify on the screen that shows the device.</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>Yes, at source, by revert. Restoring the shipped order (only the remembered map consulted) fails two of the four new tests: a_send_resolves_a_destination_that_only_discovery_can_see and discovery_wins_over_a_stale_remembered_record. With the fix, all 66 commands-lib tests and all 374 workspace tests pass. An earlier attempt that merely swapped the or_else order also failed the discovery_wins test -- so the order rule has teeth as well as the primary-source rule.</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>2026-09-28 20:22</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>Also added DiscoveryService::insert_for_test (cfg(test) only) so a test can prove get_device reads the same map the browse loop writes. The four tests: discovery alone resolves a send (the real Field state: remembered is None), discovery beats a stale address, a remembered peer survives record expiry, and a device in neither map is refused without the self-contradicting wording.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>BUG-027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>FEAT-040</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Restore appends the source machine's folder name to the destination the user typed</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Restoring the transferred workspace on the Windows laptop: the user typed E:/workspace-clone as the destination folder and the plan produced E:/workspace-clone/openshorts. The extra 'openshorts' is the project's manifest name, which is simply the last folder of the source path on the Mac (Documents/openshorts). The source machine's folder name was leaked onto the destination layout, where it means nothing, and the restore report then asked the user to go and create a folder they never named.</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>On the receiving machine, open a restored workspace, click Restore, type E:/workspace-clone as the destination for a bucket whose single project came from ~/Documents/openshorts, and inspect the plan.</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>The typed folder is the project's destination: the code lands in E:/workspace-clone, exactly as written.</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>The plan step read 'openshorts maps to E:/workspace-clone/openshorts' -- the chosen root with the source folder name appended.</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>resolve_destinations always resolved root.join(project.name). project.name comes from the source machine (the capture derives it from the selected folder), so a root the destination user chose was silently treated as a parent folder, and every bucket got a subfolder named after something local to the other machine. The reuse was deceptive: on the sending machine the name is the project folder (sensible), on a different machine's layout it is arbitrary. BUG-027 is the first restore-place failure seen on two real machines; the two-device tests all used synthetic names on one layout, so the leak never showed.</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>resolve_destinations now counts the projects per bucket: a bucket holding exactly one project uses the chosen folder itself as that project's destination (the user's typed path is the folder the code lands in -- no append, and the manifest name is not consulted at all, which also makes a solitary bucket immune to a hostile name); a bucket holding several projects nests each beneath the chosen folder via the existing safe_child gate, so collisions are avoided and nothing can escape the chosen root. Same-name collisions in a crowded bucket now emit a warning. The plan preview copy explains the rule, and per-project steps still show the exact final path before anything runs.</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>Yes. a_single_project_lands_exactly_in_the_folder_typed reproduces the user's exact case and fails on the old code (it asserted .../openshorts). Revert-verified: restoring root.join(name) for a solitary project fails that test plus a_solitary_project_ignores_a_hostile_name. 377 Rust tests, 99 vitest, tsc clean.</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>2026-09-28 20:40</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>User's decision (2026-09-28): exact folder for one project; nested only when a bucket holds several. Frontend copy in RestorePreviewScreen updated to state the rule. The laptop needs this fix for the restore side: planner.rs + RestorePreviewScreen.tsx must reach the Windows build.</t>
         </is>
       </c>
     </row>
@@ -19591,7 +20344,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L28"/>
+  <dimension ref="A1:L30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21331,6 +22084,130 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>DEC-029</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Policy takes camelCase aliases rather than a camelCase rename</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>`Policy` is deserialized from two places that use two different conventions: inside a `CaptureSelection` arriving over IPC, where the TypeScript is camelCase, and inside the manifest, which is snake_case on the wire by DEC-012.</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Blanket `rename_all = "camelCase"` (fixes input, rewrites the wire format); rename the TypeScript to snake_case (breaks the 9-place convention); per-field `alias` (accepts both, writes one); a separate boundary type (no alias risk, two types to keep in step).</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Per-field `alias` on the three multi-word fields, so both spellings deserialize and exactly one is ever written.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>A blanket rename would have appeared to work -- the capture would succeed -- while changing the manifest format for every stored and transferred manifest, which is a compatibility break in a field nothing tests. A separate type would be cleaner in principle but means two structs to keep in step forever. The alias keeps one type, accepts both spellings, and fails loudly if both are present.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>The manifest wire format is unchanged, verified by a round-trip test. The four Policy fields are the only ones needing this treatment; `clipboard` is one word and is spelled the same in both conventions, so an alias for it would have been misleading.</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>If the manifest ever gains its own versioning per field, or the IPC boundary moves off Tauri's automatic argument mapping.</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>BUG-024,FEAT-075</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>DEC-030</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>IP payloads deny unknown fields instead of ignoring them</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Serde ignores an unrecognised key by default, so a field the UI sends under a name the Rust struct does not know arrives as an empty list, not an error.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Leave the default (silent); reject the whole payload on an unknown key; log a warning and continue.</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Reject the payload.</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Silent truncation is the worst available outcome: a capture completes, reports success, and quietly omits what the user selected. The symptom points somewhere else entirely -- in BUG-024 the URLs vanished and the browser adapter looked at fault, when the cause was four functions away. A user who selects three projects and pastes two URLs cannot tell an empty list that arrived empty from one that was dropped in transit. The UI and the Rust types are hand-mirrored in two languages, so the realistic failure is a typo, and a typo should stop the capture.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>A field added in TypeScript before the Rust struct catches up now fails the command loudly instead of arriving empty. Applied to the three capture-selection types; deliberately NOT applied to `Policy`, which is also a wire format, where the manifest's own schema validation is the right mechanism and an unknown field could come from a newer sender.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>If the frontend ever needs to send fields the backend does not model, or if a version skew between machines becomes possible.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>BUG-024,FEAT-075</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix BUG-022: renumber the tracker Tasks sheet and repair its dependency columns
Rows 42-73 were TASK-031..TASK-060 duplicating the first block's numbering
(14 rows shared an ID), and 67 rows carried their dependency lists in the
Assignee column. Per the recorded decision: renumber the second block to
TASK-041..TASK-072 in row order, move the 67 lists into the Dependencies
column, and remap references (first-occurrence rule; only second-block-unique
labels change: TASK-042->056, 047->061, 048->062, 056->068). BUG-022 set to
Fixed; LOG-087 records the fix and the caveat about the bulk-populated source
of the dependency values.
</commit_message>
<xml_diff>
--- a/WorkspaceClone_Tracking.xlsx
+++ b/WorkspaceClone_Tracking.xlsx
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I83"/>
+  <dimension ref="A1:I84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4742,6 +4742,53 @@
       <c r="I83" t="inlineStr">
         <is>
           <t>build,release,dmg,deferred-note</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>LOG-087</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>2026-09-28 22:10</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>FIX</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>Project Data</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>BUG-022</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Tasks sheet renumbered and dependency columns fixed</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>BUG-022 fixed per the chosen option (second block renumbered): rows 42-73 became TASK-041..TASK-072 in row order, so all 72 task rows now have unique IDs (the 14 shared IDs are gone). The 67 dependency lists sitting in the Assignee column (38 first-block + 29 second-block rows) moved into the Dependencies column. References remapped by the first-occurrence rule: only labels whose first sheet occurrence is in the second block changed -- TASK-042-&gt;056, TASK-047-&gt;061, TASK-048-&gt;062, TASK-056-&gt;068; ambiguous labels TASK-031..040 resolve to the canonical first block and were left as written. Caveat: the dependency VALUES were bulk-populated when the sheet was built and their semantics remain the original author's intent, not a derived DAG -- but the column each chain sits in is now the one its header names. Re-verified by script asserts on 2026-09-28.</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>bug,data-quality,tasks-sheet,correction</t>
         </is>
       </c>
     </row>
@@ -11407,12 +11454,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L3" s="2" t="inlineStr">
+      <c r="L3" s="2" t="n"/>
+      <c r="M3" s="2" t="inlineStr">
         <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr"/>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
@@ -11468,12 +11515,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L4" s="2" t="inlineStr">
+      <c r="L4" s="2" t="n"/>
+      <c r="M4" s="2" t="inlineStr">
         <is>
           <t>TASK-002</t>
         </is>
       </c>
-      <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr"/>
       <c r="O4" s="2" t="inlineStr"/>
       <c r="P4" s="2" t="inlineStr"/>
@@ -11529,12 +11576,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L5" s="2" t="inlineStr">
+      <c r="L5" s="2" t="n"/>
+      <c r="M5" s="2" t="inlineStr">
         <is>
           <t>TASK-002</t>
         </is>
       </c>
-      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr"/>
       <c r="O5" s="2" t="inlineStr"/>
       <c r="P5" s="2" t="inlineStr"/>
@@ -11590,12 +11637,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L6" s="2" t="inlineStr">
+      <c r="L6" s="2" t="n"/>
+      <c r="M6" s="2" t="inlineStr">
         <is>
           <t>TASK-003, TASK-004</t>
         </is>
       </c>
-      <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr"/>
       <c r="O6" s="2" t="inlineStr"/>
       <c r="P6" s="2" t="inlineStr"/>
@@ -11651,12 +11698,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" s="2" t="inlineStr">
         <is>
           <t>TASK-005</t>
         </is>
       </c>
-      <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="inlineStr"/>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -11712,12 +11759,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" s="2" t="inlineStr">
         <is>
           <t>TASK-006</t>
         </is>
       </c>
-      <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr"/>
       <c r="O8" s="2" t="inlineStr"/>
       <c r="P8" s="2" t="inlineStr"/>
@@ -11773,12 +11820,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
+      <c r="L9" s="2" t="n"/>
+      <c r="M9" s="2" t="inlineStr">
         <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr"/>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -11834,12 +11881,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" s="2" t="inlineStr">
         <is>
           <t>TASK-008</t>
         </is>
       </c>
-      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr"/>
       <c r="O10" s="2" t="inlineStr"/>
       <c r="P10" s="2" t="inlineStr"/>
@@ -11895,12 +11942,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
+      <c r="L11" s="2" t="n"/>
+      <c r="M11" s="2" t="inlineStr">
         <is>
           <t>TASK-004</t>
         </is>
       </c>
-      <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr"/>
       <c r="O11" s="2" t="inlineStr"/>
       <c r="P11" s="2" t="inlineStr"/>
@@ -11956,12 +12003,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L12" s="2" t="n"/>
+      <c r="M12" s="2" t="inlineStr">
         <is>
           <t>TASK-010</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr"/>
       <c r="N12" s="2" t="inlineStr"/>
       <c r="O12" s="2" t="inlineStr"/>
       <c r="P12" s="2" t="inlineStr"/>
@@ -12017,12 +12064,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
+      <c r="L13" s="2" t="n"/>
+      <c r="M13" s="2" t="inlineStr">
         <is>
           <t>TASK-003</t>
         </is>
       </c>
-      <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr"/>
       <c r="O13" s="2" t="inlineStr"/>
       <c r="P13" s="2" t="inlineStr"/>
@@ -12135,12 +12182,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L15" s="2" t="inlineStr">
+      <c r="L15" s="2" t="n"/>
+      <c r="M15" s="2" t="inlineStr">
         <is>
           <t>TASK-013</t>
         </is>
       </c>
-      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr"/>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -12196,12 +12243,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
+      <c r="L16" s="2" t="n"/>
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>TASK-014</t>
         </is>
       </c>
-      <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr"/>
       <c r="O16" s="2" t="inlineStr"/>
       <c r="P16" s="2" t="inlineStr"/>
@@ -12257,12 +12304,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
+      <c r="L17" s="2" t="n"/>
+      <c r="M17" s="2" t="inlineStr">
         <is>
           <t>TASK-014</t>
         </is>
       </c>
-      <c r="M17" s="2" t="inlineStr"/>
       <c r="N17" s="2" t="inlineStr"/>
       <c r="O17" s="2" t="inlineStr"/>
       <c r="P17" s="2" t="inlineStr"/>
@@ -12318,12 +12365,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L18" s="2" t="n"/>
+      <c r="M18" s="2" t="inlineStr">
         <is>
           <t>TASK-016</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr"/>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
@@ -12379,12 +12426,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L19" s="2" t="inlineStr">
+      <c r="L19" s="2" t="n"/>
+      <c r="M19" s="2" t="inlineStr">
         <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr"/>
       <c r="O19" s="2" t="inlineStr"/>
       <c r="P19" s="2" t="inlineStr"/>
@@ -12440,12 +12487,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L20" s="2" t="inlineStr">
+      <c r="L20" s="2" t="n"/>
+      <c r="M20" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr"/>
       <c r="O20" s="2" t="inlineStr"/>
       <c r="P20" s="2" t="inlineStr"/>
@@ -12501,12 +12548,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L21" s="2" t="inlineStr">
+      <c r="L21" s="2" t="n"/>
+      <c r="M21" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr"/>
       <c r="O21" s="2" t="inlineStr"/>
       <c r="P21" s="2" t="inlineStr"/>
@@ -12562,12 +12609,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L22" s="2" t="inlineStr">
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="inlineStr">
         <is>
           <t>TASK-020</t>
         </is>
       </c>
-      <c r="M22" s="2" t="inlineStr"/>
       <c r="N22" s="2" t="inlineStr"/>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
@@ -12623,12 +12670,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L23" s="2" t="inlineStr">
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr"/>
       <c r="O23" s="2" t="inlineStr"/>
       <c r="P23" s="2" t="inlineStr"/>
@@ -12684,12 +12731,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L24" s="2" t="inlineStr">
+      <c r="L24" s="2" t="n"/>
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr"/>
       <c r="O24" s="2" t="inlineStr"/>
       <c r="P24" s="2" t="inlineStr"/>
@@ -12745,12 +12792,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="L25" s="2" t="n"/>
+      <c r="M25" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr"/>
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
@@ -12806,12 +12853,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L26" s="2" t="inlineStr">
+      <c r="L26" s="2" t="n"/>
+      <c r="M26" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M26" s="2" t="inlineStr"/>
       <c r="N26" s="2" t="inlineStr"/>
       <c r="O26" s="2" t="inlineStr"/>
       <c r="P26" s="2" t="inlineStr"/>
@@ -12867,12 +12914,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L27" s="2" t="inlineStr">
+      <c r="L27" s="2" t="n"/>
+      <c r="M27" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr"/>
       <c r="O27" s="2" t="inlineStr"/>
       <c r="P27" s="2" t="inlineStr"/>
@@ -12928,12 +12975,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L28" s="2" t="inlineStr">
+      <c r="L28" s="2" t="n"/>
+      <c r="M28" s="2" t="inlineStr">
         <is>
           <t>TASK-018</t>
         </is>
       </c>
-      <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr"/>
       <c r="P28" s="2" t="inlineStr"/>
@@ -12989,12 +13036,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L29" s="2" t="inlineStr">
+      <c r="L29" s="2" t="n"/>
+      <c r="M29" s="2" t="inlineStr">
         <is>
           <t>TASK-023..027</t>
         </is>
       </c>
-      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr"/>
       <c r="O29" s="2" t="inlineStr"/>
       <c r="P29" s="2" t="inlineStr"/>
@@ -13050,12 +13097,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L30" s="2" t="inlineStr">
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="inlineStr">
         <is>
           <t>TASK-014</t>
         </is>
       </c>
-      <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr"/>
       <c r="O30" s="2" t="inlineStr"/>
       <c r="P30" s="2" t="inlineStr"/>
@@ -13111,12 +13158,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L31" s="2" t="inlineStr">
+      <c r="L31" s="2" t="n"/>
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>TASK-029</t>
         </is>
       </c>
-      <c r="M31" s="2" t="inlineStr"/>
       <c r="N31" s="2" t="inlineStr"/>
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
@@ -13172,12 +13219,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="L32" s="2" t="n"/>
+      <c r="M32" s="2" t="inlineStr">
         <is>
           <t>TASK-030</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr"/>
       <c r="O32" s="2" t="inlineStr"/>
       <c r="P32" s="2" t="inlineStr"/>
@@ -13233,12 +13280,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L33" s="2" t="inlineStr">
+      <c r="L33" s="2" t="n"/>
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>TASK-030</t>
         </is>
       </c>
-      <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr"/>
       <c r="O33" s="2" t="inlineStr"/>
       <c r="P33" s="2" t="inlineStr"/>
@@ -13294,12 +13341,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L34" s="2" t="n"/>
+      <c r="M34" s="2" t="inlineStr">
         <is>
           <t>TASK-030</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr"/>
       <c r="O34" s="2" t="inlineStr"/>
       <c r="P34" s="2" t="inlineStr"/>
@@ -13355,12 +13402,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L35" s="2" t="inlineStr">
+      <c r="L35" s="2" t="n"/>
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>TASK-030</t>
         </is>
       </c>
-      <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr"/>
       <c r="O35" s="2" t="inlineStr"/>
       <c r="P35" s="2" t="inlineStr"/>
@@ -13416,12 +13463,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L36" s="2" t="inlineStr">
+      <c r="L36" s="2" t="n"/>
+      <c r="M36" s="2" t="inlineStr">
         <is>
           <t>TASK-029</t>
         </is>
       </c>
-      <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr"/>
       <c r="O36" s="2" t="inlineStr"/>
       <c r="P36" s="2" t="inlineStr"/>
@@ -13477,12 +13524,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L37" s="2" t="inlineStr">
+      <c r="L37" s="2" t="n"/>
+      <c r="M37" s="2" t="inlineStr">
         <is>
           <t>TASK-029</t>
         </is>
       </c>
-      <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr"/>
       <c r="O37" s="2" t="inlineStr"/>
       <c r="P37" s="2" t="inlineStr"/>
@@ -13538,12 +13585,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L38" s="2" t="inlineStr">
+      <c r="L38" s="2" t="n"/>
+      <c r="M38" s="2" t="inlineStr">
         <is>
           <t>TASK-036</t>
         </is>
       </c>
-      <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr"/>
       <c r="O38" s="2" t="inlineStr"/>
       <c r="P38" s="2" t="inlineStr"/>
@@ -13599,12 +13646,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L39" s="2" t="inlineStr">
+      <c r="L39" s="2" t="n"/>
+      <c r="M39" s="2" t="inlineStr">
         <is>
           <t>TASK-035</t>
         </is>
       </c>
-      <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr"/>
       <c r="O39" s="2" t="inlineStr"/>
       <c r="P39" s="2" t="inlineStr"/>
@@ -13660,12 +13707,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L40" s="2" t="inlineStr">
+      <c r="L40" s="2" t="n"/>
+      <c r="M40" s="2" t="inlineStr">
         <is>
           <t>TASK-037</t>
         </is>
       </c>
-      <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr"/>
       <c r="O40" s="2" t="inlineStr"/>
       <c r="P40" s="2" t="inlineStr"/>
@@ -13721,12 +13768,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L41" s="2" t="inlineStr">
+      <c r="L41" s="2" t="n"/>
+      <c r="M41" s="2" t="inlineStr">
         <is>
           <t>TASK-033, TASK-018</t>
         </is>
       </c>
-      <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr"/>
       <c r="O41" s="2" t="inlineStr"/>
       <c r="P41" s="2" t="inlineStr"/>
@@ -13735,7 +13782,7 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>TASK-031</t>
+          <t>TASK-041</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
@@ -13782,12 +13829,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L42" s="2" t="inlineStr">
+      <c r="L42" s="2" t="n"/>
+      <c r="M42" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr"/>
       <c r="O42" s="2" t="inlineStr"/>
       <c r="P42" s="2" t="inlineStr"/>
@@ -13796,7 +13843,7 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>TASK-032</t>
+          <t>TASK-042</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
@@ -13843,12 +13890,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L43" s="2" t="inlineStr">
+      <c r="L43" s="2" t="n"/>
+      <c r="M43" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr"/>
       <c r="O43" s="2" t="inlineStr"/>
       <c r="P43" s="2" t="inlineStr"/>
@@ -13857,7 +13904,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>TASK-033</t>
+          <t>TASK-043</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
@@ -13904,12 +13951,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L44" s="2" t="inlineStr">
+      <c r="L44" s="2" t="n"/>
+      <c r="M44" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr"/>
       <c r="O44" s="2" t="inlineStr"/>
       <c r="P44" s="2" t="inlineStr"/>
@@ -13918,7 +13965,7 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>TASK-034</t>
+          <t>TASK-044</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
@@ -13965,12 +14012,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L45" s="2" t="inlineStr">
+      <c r="L45" s="2" t="n"/>
+      <c r="M45" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr"/>
       <c r="O45" s="2" t="inlineStr"/>
       <c r="P45" s="2" t="inlineStr"/>
@@ -13979,7 +14026,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>TASK-034</t>
+          <t>TASK-045</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
@@ -14026,12 +14073,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L46" s="2" t="inlineStr">
+      <c r="L46" s="2" t="n"/>
+      <c r="M46" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr"/>
       <c r="O46" s="2" t="inlineStr"/>
       <c r="P46" s="2" t="inlineStr"/>
@@ -14040,7 +14087,7 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>TASK-035</t>
+          <t>TASK-046</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
@@ -14087,12 +14134,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L47" s="2" t="inlineStr">
+      <c r="L47" s="2" t="n"/>
+      <c r="M47" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr"/>
       <c r="O47" s="2" t="inlineStr"/>
       <c r="P47" s="2" t="inlineStr"/>
@@ -14101,7 +14148,7 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>TASK-036</t>
+          <t>TASK-047</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
@@ -14148,12 +14195,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L48" s="2" t="inlineStr">
+      <c r="L48" s="2" t="n"/>
+      <c r="M48" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr"/>
       <c r="O48" s="2" t="inlineStr"/>
       <c r="P48" s="2" t="inlineStr"/>
@@ -14162,7 +14209,7 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>TASK-036</t>
+          <t>TASK-048</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
@@ -14209,12 +14256,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L49" s="2" t="inlineStr">
+      <c r="L49" s="2" t="n"/>
+      <c r="M49" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr"/>
       <c r="O49" s="2" t="inlineStr"/>
       <c r="P49" s="2" t="inlineStr"/>
@@ -14223,7 +14270,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>TASK-037</t>
+          <t>TASK-049</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
@@ -14270,12 +14317,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L50" s="2" t="inlineStr">
+      <c r="L50" s="2" t="n"/>
+      <c r="M50" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr"/>
       <c r="O50" s="2" t="inlineStr"/>
       <c r="P50" s="2" t="inlineStr"/>
@@ -14284,7 +14331,7 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>TASK-037</t>
+          <t>TASK-050</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
@@ -14331,12 +14378,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L51" s="2" t="inlineStr">
+      <c r="L51" s="2" t="n"/>
+      <c r="M51" s="2" t="inlineStr">
         <is>
           <t>TASK-037</t>
         </is>
       </c>
-      <c r="M51" s="2" t="inlineStr"/>
       <c r="N51" s="2" t="inlineStr"/>
       <c r="O51" s="2" t="inlineStr"/>
       <c r="P51" s="2" t="inlineStr"/>
@@ -14345,7 +14392,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>TASK-038</t>
+          <t>TASK-051</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
@@ -14392,12 +14439,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L52" s="2" t="inlineStr">
+      <c r="L52" s="2" t="n"/>
+      <c r="M52" s="2" t="inlineStr">
         <is>
           <t>TASK-037</t>
         </is>
       </c>
-      <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr"/>
       <c r="O52" s="2" t="inlineStr"/>
       <c r="P52" s="2" t="inlineStr"/>
@@ -14406,7 +14453,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>TASK-038</t>
+          <t>TASK-052</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
@@ -14453,12 +14500,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L53" s="2" t="inlineStr">
+      <c r="L53" s="2" t="n"/>
+      <c r="M53" s="2" t="inlineStr">
         <is>
           <t>TASK-037</t>
         </is>
       </c>
-      <c r="M53" s="2" t="inlineStr"/>
       <c r="N53" s="2" t="inlineStr"/>
       <c r="O53" s="2" t="inlineStr"/>
       <c r="P53" s="2" t="inlineStr"/>
@@ -14467,7 +14514,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>TASK-039</t>
+          <t>TASK-053</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
@@ -14514,12 +14561,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L54" s="2" t="inlineStr">
+      <c r="L54" s="2" t="n"/>
+      <c r="M54" s="2" t="inlineStr">
         <is>
           <t>TASK-038</t>
         </is>
       </c>
-      <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr"/>
       <c r="O54" s="2" t="inlineStr"/>
       <c r="P54" s="2" t="inlineStr"/>
@@ -14528,7 +14575,7 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>TASK-040</t>
+          <t>TASK-054</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
@@ -14575,12 +14622,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L55" s="2" t="inlineStr">
+      <c r="L55" s="2" t="n"/>
+      <c r="M55" s="2" t="inlineStr">
         <is>
           <t>TASK-038</t>
         </is>
       </c>
-      <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr"/>
       <c r="O55" s="2" t="inlineStr"/>
       <c r="P55" s="2" t="inlineStr"/>
@@ -14589,7 +14636,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>TASK-041</t>
+          <t>TASK-055</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
@@ -14636,12 +14683,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L56" s="2" t="inlineStr">
+      <c r="L56" s="2" t="n"/>
+      <c r="M56" s="2" t="inlineStr">
         <is>
           <t>TASK-038</t>
         </is>
       </c>
-      <c r="M56" s="2" t="inlineStr"/>
       <c r="N56" s="2" t="inlineStr"/>
       <c r="O56" s="2" t="inlineStr"/>
       <c r="P56" s="2" t="inlineStr"/>
@@ -14650,7 +14697,7 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>TASK-042</t>
+          <t>TASK-056</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
@@ -14697,12 +14744,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L57" s="2" t="inlineStr">
+      <c r="L57" s="2" t="n"/>
+      <c r="M57" s="2" t="inlineStr">
         <is>
           <t>TASK-037</t>
         </is>
       </c>
-      <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr"/>
       <c r="O57" s="2" t="inlineStr"/>
       <c r="P57" s="2" t="inlineStr"/>
@@ -14711,7 +14758,7 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>TASK-043</t>
+          <t>TASK-057</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
@@ -14758,12 +14805,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L58" s="2" t="inlineStr">
-        <is>
-          <t>TASK-042</t>
-        </is>
-      </c>
-      <c r="M58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="n"/>
+      <c r="M58" s="2" t="inlineStr">
+        <is>
+          <t>TASK-056</t>
+        </is>
+      </c>
       <c r="N58" s="2" t="inlineStr"/>
       <c r="O58" s="2" t="inlineStr"/>
       <c r="P58" s="2" t="inlineStr"/>
@@ -14772,7 +14819,7 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>TASK-044</t>
+          <t>TASK-058</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
@@ -14819,12 +14866,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L59" s="2" t="inlineStr">
+      <c r="L59" s="2" t="n"/>
+      <c r="M59" s="2" t="inlineStr">
         <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="M59" s="2" t="inlineStr"/>
       <c r="N59" s="2" t="inlineStr"/>
       <c r="O59" s="2" t="inlineStr"/>
       <c r="P59" s="2" t="inlineStr"/>
@@ -14833,7 +14880,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>TASK-045</t>
+          <t>TASK-059</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
@@ -14880,12 +14927,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L60" s="2" t="inlineStr">
+      <c r="L60" s="2" t="n"/>
+      <c r="M60" s="2" t="inlineStr">
         <is>
           <t>TASK-032</t>
         </is>
       </c>
-      <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr"/>
       <c r="O60" s="2" t="inlineStr"/>
       <c r="P60" s="2" t="inlineStr"/>
@@ -14894,7 +14941,7 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>TASK-046</t>
+          <t>TASK-060</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
@@ -14941,12 +14988,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L61" s="2" t="inlineStr">
+      <c r="L61" s="2" t="n"/>
+      <c r="M61" s="2" t="inlineStr">
         <is>
           <t>TASK-022</t>
         </is>
       </c>
-      <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr"/>
       <c r="O61" s="2" t="inlineStr"/>
       <c r="P61" s="2" t="inlineStr"/>
@@ -14955,7 +15002,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>TASK-047</t>
+          <t>TASK-061</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
@@ -15002,12 +15049,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L62" s="2" t="inlineStr">
+      <c r="L62" s="2" t="n"/>
+      <c r="M62" s="2" t="inlineStr">
         <is>
           <t>TASK-028</t>
         </is>
       </c>
-      <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr"/>
       <c r="O62" s="2" t="inlineStr"/>
       <c r="P62" s="2" t="inlineStr"/>
@@ -15016,7 +15063,7 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>TASK-048</t>
+          <t>TASK-062</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
@@ -15063,12 +15110,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L63" s="2" t="inlineStr">
+      <c r="L63" s="2" t="n"/>
+      <c r="M63" s="2" t="inlineStr">
         <is>
           <t>TASK-039</t>
         </is>
       </c>
-      <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="2" t="inlineStr"/>
       <c r="O63" s="2" t="inlineStr"/>
       <c r="P63" s="2" t="inlineStr"/>
@@ -15077,7 +15124,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>TASK-050</t>
+          <t>TASK-063</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
@@ -15124,12 +15171,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L64" s="2" t="inlineStr">
+      <c r="L64" s="2" t="n"/>
+      <c r="M64" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M64" s="2" t="inlineStr"/>
       <c r="N64" s="2" t="inlineStr"/>
       <c r="O64" s="2" t="inlineStr"/>
       <c r="P64" s="2" t="inlineStr"/>
@@ -15138,7 +15185,7 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>TASK-052</t>
+          <t>TASK-064</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
@@ -15185,12 +15232,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L65" s="2" t="inlineStr">
+      <c r="L65" s="2" t="n"/>
+      <c r="M65" s="2" t="inlineStr">
         <is>
           <t>TASK-040</t>
         </is>
       </c>
-      <c r="M65" s="2" t="inlineStr"/>
       <c r="N65" s="2" t="inlineStr"/>
       <c r="O65" s="2" t="inlineStr"/>
       <c r="P65" s="2" t="inlineStr"/>
@@ -15199,7 +15246,7 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>TASK-053</t>
+          <t>TASK-065</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
@@ -15246,12 +15293,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L66" s="2" t="inlineStr">
-        <is>
-          <t>TASK-047</t>
-        </is>
-      </c>
-      <c r="M66" s="2" t="inlineStr"/>
+      <c r="L66" s="2" t="n"/>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>TASK-061</t>
+        </is>
+      </c>
       <c r="N66" s="2" t="inlineStr"/>
       <c r="O66" s="2" t="inlineStr"/>
       <c r="P66" s="2" t="inlineStr"/>
@@ -15260,7 +15307,7 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>TASK-054</t>
+          <t>TASK-066</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
@@ -15307,12 +15354,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L67" s="2" t="inlineStr">
-        <is>
-          <t>TASK-048</t>
-        </is>
-      </c>
-      <c r="M67" s="2" t="inlineStr"/>
+      <c r="L67" s="2" t="n"/>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>TASK-062</t>
+        </is>
+      </c>
       <c r="N67" s="2" t="inlineStr"/>
       <c r="O67" s="2" t="inlineStr"/>
       <c r="P67" s="2" t="inlineStr"/>
@@ -15321,7 +15368,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>TASK-055</t>
+          <t>TASK-067</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
@@ -15368,12 +15415,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L68" s="2" t="inlineStr">
+      <c r="L68" s="2" t="n"/>
+      <c r="M68" s="2" t="inlineStr">
         <is>
           <t>TASK-001</t>
         </is>
       </c>
-      <c r="M68" s="2" t="inlineStr"/>
       <c r="N68" s="2" t="inlineStr"/>
       <c r="O68" s="2" t="inlineStr"/>
       <c r="P68" s="2" t="inlineStr"/>
@@ -15382,7 +15429,7 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>TASK-056</t>
+          <t>TASK-068</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
@@ -15429,12 +15476,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L69" s="2" t="inlineStr">
+      <c r="L69" s="2" t="n"/>
+      <c r="M69" s="2" t="inlineStr">
         <is>
           <t>TASK-014</t>
         </is>
       </c>
-      <c r="M69" s="2" t="inlineStr"/>
       <c r="N69" s="2" t="inlineStr"/>
       <c r="O69" s="2" t="inlineStr"/>
       <c r="P69" s="2" t="inlineStr"/>
@@ -15443,7 +15490,7 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>TASK-057</t>
+          <t>TASK-069</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
@@ -15490,12 +15537,12 @@
           <t>2026-09-26</t>
         </is>
       </c>
-      <c r="L70" s="2" t="inlineStr">
-        <is>
-          <t>TASK-056</t>
-        </is>
-      </c>
-      <c r="M70" s="2" t="inlineStr"/>
+      <c r="L70" s="2" t="n"/>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>TASK-068</t>
+        </is>
+      </c>
       <c r="N70" s="2" t="inlineStr"/>
       <c r="O70" s="2" t="inlineStr"/>
       <c r="P70" s="2" t="inlineStr"/>
@@ -15504,7 +15551,7 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>TASK-058</t>
+          <t>TASK-070</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
@@ -15557,7 +15604,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>TASK-059</t>
+          <t>TASK-071</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
@@ -15610,7 +15657,7 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>TASK-060</t>
+          <t>TASK-072</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
@@ -17635,7 +17682,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Not Fixed</t>
+          <t>Fixed</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -17660,15 +17707,20 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Not fixed. The column offset is mechanical and safe to correct, but the duplicate IDs are not, and repairing them requires deciding what each dependency reference means. References are genuinely split: row 70's 'TASK-056' points at a task in the second batch (Named Destination Roots, which Cross-Platform Path Translation sensibly follows), while row 60's 'TASK-032' points at one in the first batch (Device Management UI, which a Devices screen sensibly follows). A nearest-match rule resolves the first correctly and the second wrongly, and the two cannot be told apart from the data alone. Renumbering 32 rows on a coin flip would silently corrupt the dependency graph further.</t>
+          <t>Rows 42-73 renumbered TASK-031..TASK-060 -&gt; TASK-041..TASK-072 in row order, so every ID is unique. The 67 dependency lists sitting in the Assignee column moved to the Dependencies column (38 first-block + 29 second-block rows; the sheet already had 3 in the right column). References remapped by the first-occurrence rule: labels only present in the second block (TASK-041..060) resolve to their renumbered first occurrence; ambiguous labels present in both blocks resolve to the canonical first block and stay as written.</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Diagnosis verified: the duplicate IDs, the two numbering batches and the 67 misplaced dependency cells were all read directly out of the workbook. The fix is explicitly not attempted.</t>
+          <t>ID uniqueness, column placement and reference remap all re-checked by script asserts on 2026-09-28. Residual caveat recorded in LOG-087: the dependency VALUES were bulk-populated and their semantics remain the author's intent, not a derived DAG.</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
+        <is>
+          <t>2026-09-28</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
         <is>
           <t>2026-09-28</t>
         </is>
@@ -20766,7 +20818,6 @@
           <t>Workspace Clone_0.1.0_aarch64.dmg, 8.2 MB, plus the .app bundle. Ad-hoc signed (signingIdentity '-'). beforeBuildCommand ran npm run build first. One deprecation warning from tauri-build about STATIC_VCRUNTIME (release-profile only, Windows CRT config, not from any crate in the workspace); see LOG-086.</t>
         </is>
       </c>
-      <c r="K29" t="inlineStr"/>
       <c r="L29" t="inlineStr">
         <is>
           <t>src-tauri/target/release/bundle/dmg/Workspace Clone_0.1.0_aarch64.dmg</t>

</xml_diff>

<commit_message>
tracker: BUG-029 fixed, RUN-030, LOG-089 (arrival list refresh + capture analysis)
</commit_message>
<xml_diff>
--- a/WorkspaceClone_Tracking.xlsx
+++ b/WorkspaceClone_Tracking.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>405 Rust tests (12 of them two-device end-to-end across a real socket; 13 in the new files crate; 11 connect-candidate and dual-stack listener tests in the network crate), 99 frontend tests, 0 build warnings, command-surface parity clean at 44/44</t>
+          <t>405 Rust tests (12 of them two-device end-to-end across a real socket; 13 in the new files crate; 11 connect-candidate and dual-stack listener tests in the network crate), 100 frontend tests, 0 build warnings, command-surface parity clean at 44/44</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-28 23:10</t>
+          <t>2026-09-29 10:30</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I85"/>
+  <dimension ref="A1:I86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4836,6 +4836,53 @@
       <c r="I85" t="inlineStr">
         <is>
           <t>bug,network,ipv6,link-local,connect-fix</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>LOG-089</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:30</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>FIX + ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>Frontend / Workspaces Screen</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>BUG-029,FEAT-051</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>BUG-029 fixed; Windows-&gt;Mac retest analysed: arrival correct, capture was near-empty</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>BUG-029 resolved in WorkspacesScreen.tsx: a newly-seen accepted arrival in the incoming-transfers poll now invalidates ['workspaces'], so a workspace that arrives while the list is open appears without a menu change. New vitest pins it; suite is now 100 frontend tests, tsc clean. On the hardware retest, the green banner rendered 'Testing Window - Mac' and the Mac DB stores it with source BISWAJITA - so the reported empty-looking banner was not reproducible from current data and needs the screenshot. The 'restore shows nothing' report was root-caused on the sender side: the unsealed received manifest for bbb38119 has projects=0 and one optional terminal-session application, and no workspace_files row exists - the Windows capture selected no projects, so no file archive was ever carried and the restore plan legitimately has nothing. DEVELOPER_GUIDE gains a 'received workspace restores as nothing selected' entry pointing at the sender's project scan (default roots ~/projects, ~/Documents) and Settings -&gt; Project locations. Next: user to reattach the two screenshots and on Windows to set project roots, tick projects, re-capture and re-send.</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>frontend,arrival,workspaces-list,bug,analysis,restore,capture</t>
         </is>
       </c>
     </row>
@@ -15765,7 +15812,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -18302,6 +18349,93 @@
       <c r="Q29" t="inlineStr">
         <is>
           <t>The reported address as copied reads fe80::f727:abc9:2280:4f3:54108, whose final group has five hex digits; std rejects it and only the kernel resolver accepts it -- the fix does not depend on the exact spelling, and unparseable entries are skipped in favour of the addresses that do parse. Laptop retest steps: git pull, rebuild + reinstall the .exe on Windows, then send Mac-&gt;Windows and Windows-&gt;Mac.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>BUG-029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>FEAT-051</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>A workspace that arrives while the Workspaces screen is open stays invisible in the list until the user switches menus</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Post-BUG-028 retest on hardware. Sending 'Testing Window - Mac' from the paired Windows laptop (BISWAJITA) to the Mac completed: the green arrival banner appeared at the top of the Workspaces screen, but the new workspace was not in the list below. Navigating to another menu and back made it appear. The workspace is stored correctly by the backend; the window just never asked for the list again.</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>Receive a workspace (any direction) while sitting on the Workspaces screen with the list already fetched, then look at the list without navigating.</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>The accepted workspace appears in the list as soon as it arrives.</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>The green banner appeared but the workspace only materialised in the list after a manual navigation that remounted the screen.</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>The workspaces query (['workspaces']) is fetched on mount and was never invalidated. The arrivals poll (['incoming-transfers'], ARRIVALS_POLL_MS) is the channel that proves something arrived, so a UI with no listener meant the list kept serving its pre-arrival snapshot until something forced a refetch.</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>WorkspacesScreen now watches the arrivals poll for a previously unseen *accepted* arrival with a workspace id and invalidates ['workspaces'] at that moment, so the list refetches right away. Seen transfer ids are tracked in a ref so a restart or re-render does not re-invalidate; refusals do not invalidate (nothing was stored).</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>Yes, at source. New vitest 'puts a workspace that arrived after load into the list without a remount' drives the poll to flip from empty to a landed arrival and asserts list_workspaces is invoked again and the new workspace renders with no navigation. Suite: 100 frontend tests (was 99), tsc --noEmit clean.</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>Found by inspecting the live Mac DB after the retest: workspace bbb38119 (name 'Testing Window - Mac') was stored correctly with source BISWAJITA, so the data was always there and only the window's cache was stale. Same fix covers the reverse direction.</t>
         </is>
       </c>
     </row>
@@ -19124,7 +19258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N30"/>
+  <dimension ref="A1:N31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21023,6 +21157,64 @@
       <c r="N30" t="inlineStr">
         <is>
           <t>Companion gate: cargo build --workspace is warning-free (the only warning anywhere is a pre-existing unused-mut in wire.rs test code, invisible to the build gate). Frontend untouched, so 99 vitest + tsc stay as RUN-026/027 state.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>RUN-030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Frontend / BUG-029</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>npx vitest run &amp;&amp; npx tsc --noEmit</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:02</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2026-09-29 10:03</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>20</v>
+      </c>
+      <c r="I31" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>100 frontend tests passed across 6 files, including the new arrival-refreshes-the-list test. tsc --noEmit is clean. receive.test.tsx grew 19 -&gt; 20.</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>Companion screen for BUG-029: the two 'polling' tests together pin both halves of an arrival - the banner appears (already covered) and now the list refetches without a remount. No Rust changes in this session.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix BUG-037: git working-tree changes travel as a patch, so restore changes one file not 146
Capture now records a dirty repo's delta as a git-applyable patch (`git diff HEAD
--binary` plus one new-file hunk per untracked, non-ignored file, denylist
applied, source index never mutated) in new optional `GitInfo.patch`. Restore
plans `git-apply-<id>` instead of whole-tree extraction for patched projects;
the git adapter applies with `git apply --binary --whitespace=nowarn`. A patch
that cannot apply (base mismatch) reports `git checkout <commit>` as its remedy.
`dirty_state_captured` now means the delta contents were captured.

Tracker: BUG-037, RUN-033, LOG-091, DEC-034, Overview + FEAT-014/042/079 notes.
</commit_message>
<xml_diff>
--- a/WorkspaceClone_Tracking.xlsx
+++ b/WorkspaceClone_Tracking.xlsx
@@ -805,7 +805,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>408 Rust tests (12 of them two-device end-to-end across a real socket; 7 in the db crate including both cascade-delete paths; 13 in the new files crate; 11 connect-candidate and dual-stack listener tests in the network crate), 102 frontend tests, 0 build warnings, command-surface parity clean at 44/44</t>
+          <t>419 Rust tests (was 408). The +11: 6 git-adapter tests proving a dirty worktree captures as an appliable patch and restore applies exactly that delta (`git status` matches), a mismatched base reports the checkout remedy, the denylist keeps secrets out of the patch, and a clean worktree carries no patch; 2 planner tests for the extract-skip on patched projects; 1 two-device e2e sending a dirty repo's delta over a real socket and restoring it to exactly 'M note.txt' + '?? new.txt'; 102 frontend tests; 0 build warnings.</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -815,7 +815,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>2026-09-29 23:45</t>
+          <t>2026-09-30 10:30</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -835,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:I88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4930,6 +4930,53 @@
       <c r="I87" t="inlineStr">
         <is>
           <t>frontend,backend,serde,wire-shape,arrival,delete,devices,bug,analysis</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>LOG-091</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>2026-09-30 10:30</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>FIX + ANALYSIS</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Backend / Adapters + Restore</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>BUG-037</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Git working-tree changes now travel as a patch, so restore changes one file instead of 146</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Capture records the dirty worktree's delta: `git diff HEAD --binary` (staged+unstaged net) plus a `git diff --no-index /dev/null &lt;file&gt;` new-file hunk per untracked, non-ignored file, filtering through the snapshot denylist and never mutating the user's index (no `git add -N`). The delta rides in new optional `GitInfo.patch` (serde default, backward compatible; the old honest lies -- dirty_state_captured always false -- are retired). Restore: patched projects skip whole-tree extraction and get a `git-apply-&lt;id&gt;` step run by the git adapter with `git apply --binary --whitespace=nowarn` from a temp patch file; a patch that cannot apply (base mismatch) is a Manual step reading 'git checkout &lt;source_commit&gt;', never a silent drop. Three bugs worth remembering: `git diff --no-index` exits 1 when files differ, so the capture must accept exit 1 or drop every untracked hunk; `str::trim` on the patch strips the final hunk line's newline and git rejects the patch as corrupt at that line; `ls-files` must use `-z` or the whole listing comes back as one newline-swallowing entry. Verified end to end: adapter capture-to-apply round trips, planner extract-skip, and a real two-device socket transfer whose restored checkout shows exactly the source's delta.</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>bug,git,patch,restore,delta,transfer,analysis</t>
         </is>
       </c>
     </row>
@@ -6715,7 +6762,11 @@
           <t>Per blueprint §11</t>
         </is>
       </c>
-      <c r="P15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Git Adapter now captures the dirty worktree as a git-applyable patch (GitInfo.patch) and applies it on restore via `git apply --binary`; the whole-tree overwrite for dirty repos is gone. 2026-09-30, BUG-037.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -8623,7 +8674,11 @@
           <t>Per blueprint §10.4</t>
         </is>
       </c>
-      <c r="P43" s="2" t="inlineStr"/>
+      <c r="P43" s="2" t="inlineStr">
+        <is>
+          <t>Git Safe Restore: patched projects restore via a git-apply step instead of whole-tree extraction, so the destination's `git status` shows exactly the source's uncommitted delta. 2026-09-30, BUG-037.</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -11288,7 +11343,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>ExtractFiles is a distinct RestoreActionType, so the preview and report render and gate it like any other step instead of it being a hidden side effect.</t>
+          <t>ExtractFiles is a distinct RestoreActionType, so the preview and report render and gate it like any other step instead of it being a hidden side effect. | Restore extracts only for projects without a captured git patch (clean repos keep the archive copy); dirty repos apply their delta instead. 2026-09-30, BUG-037.</t>
         </is>
       </c>
     </row>
@@ -15859,7 +15914,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q37"/>
+  <dimension ref="A1:Q38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -19057,6 +19112,88 @@
       <c r="P37" t="inlineStr">
         <is>
           <t>Backend verified by the new db-crate cascade test (peer's workspaces and records removed, local captures untouched). UI verified in the rebuilt app: single delete button, no Revoke, list shows only the paired laptop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>BUG-037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>FEAT-014,FEAT-042,FEAT-079</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Restore of a dirty git clone rewrote the whole tree: 146 files for one change</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>A workspace whose project is a git checkout with uncommitted changes was restored by overwriting the whole tree at the destination, so `git status` there listed every tracked file as modified. The user's real delta was one file; the restore produced 146. Reported as the transfer/restore follow-up: 'make sure to take git changes using the patch'.</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Capture a workspace that includes a dirty git repo (one modified tracked file is enough), restore it into a same-commit clone, and run `git status --short` there.</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>`git status --short` at the destination shows exactly the source's uncommitted delta (one file), nothing more.</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>`git status --short` listed every tracked file as modified (146 files): the whole tree had been extracted over the checkout.</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>The file archive does not carry file modes, and restore's extract_project writes every file with default permissions, so executable files in a same-commit checkout reported mode changes en masse. The dirty state had explicitly never been captured (dirty_state_captured was always false), so there was no way to reproduce the delta on the other side.</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Capture now records the worktree delta as a git-applyable patch: `git diff HEAD --binary` (staged + unstaged net) plus one `git diff --no-index /dev/null &lt;file&gt;` new-file hunk per untracked, non-ignored file, with the snapshot denylist applied and the source index never mutated (no `git add -N`). The patch travels in new optional `GitInfo.patch`. For patched projects the planner plans `git-apply-&lt;id&gt;` (adapter git, required false) and skips whole-tree extraction; the adapter applies via `git apply --binary --whitespace=nowarn` from a temp patch file, reporting `git checkout &lt;source_commit&gt;` as the remedy when the patch does not apply. A clean repo -- or one whose delta could not be captured -- keeps the old whole-tree copy.</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>All suites green: 419 Rust tests (6 new adapter round-trip tests on real repos -- capture-to-apply gives exact `git status`, denylist respected, clean repo has no patch, mismatched base reports the remedy -- plus 2 new planner tests for the extract-skip and 1 new two-device e2e proving the patch survives the real socket transfer and restores to the exact change), 102 frontend tests, tsc --noEmit clean, 0 build warnings.</t>
         </is>
       </c>
     </row>
@@ -19879,7 +20016,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N33"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -21952,6 +22089,64 @@
       <c r="N33" t="inlineStr">
         <is>
           <t>Full validation on real hardware and data. One live end-to-end banner check remains impossible from this machine (needs a new Windows-side send); covered by the Rust e2e + wire-shape tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RUN-033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Test</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Rust + Frontend suites / BUG-037 git patch transport</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>cargo test &amp;&amp; npx tsc --noEmit &amp;&amp; npx vitest run</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>2026-09-30 10:10</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2026-09-30 10:30</t>
+        </is>
+      </c>
+      <c r="H34" t="n">
+        <v>480</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>419 Rust tests passed (was 408): 6 new adapter tests capture a dirty worktree as a patch, apply it to an identical clone and assert `git status ` shows exactly the source delta; a mismatched-base clone reports 'git checkout &lt;commit&gt;' as a Manual remedy; the denylist keeps .env and node_modules out of the patch; a clean worktree captures no patch; plan_restore emits git-apply only when a delta exists. 2 new planner tests (patched project restores via git-apply with no extract-files step; clean project keeps the tree copy). 1 new two-device e2e: a dirty repo's delta survives the real socket + sealing round trip and restores to exactly [' M note.txt', '?? new.txt']. tsc --noEmit clean, 102 frontend tests passed, 0 build warnings.</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>One follow-up remains out of reach from this machine: a true live transfer with the Windows laptop (requires the user to send). Covered by the Rust e2e + adapter round-trip tests.</t>
         </is>
       </c>
     </row>
@@ -22659,7 +22854,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -24709,6 +24904,68 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>DEC-034</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>2026-09-30</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>A dirty git worktree travels as a `git apply`-able patch; restore applies it instead of overwriting the tree</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Capturing a workspace whose project is a dirty git clone and extracting the whole tree at restore made `git status` on the destination list every tracked file as modified (146 files for a one-file change): the archive carries no file modes, and the baseline at the destination may differ.</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Overwrite the tree as before; capture only the dirty flag (status quo); ship the patch and apply it at restore</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Record `git diff HEAD --binary` plus one new-file hunk per untracked, non-ignored file in the manifest (`GitInfo.patch`); planner plans `git-apply-&lt;id&gt;` and skips extraction for patched projects; the git adapter applies with `git apply --binary --whitespace=nowarn`</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>The delta is the honest thing to move: it is small, it is exactly what the user changed, and git apply's path validation keeps every write inside the chosen destination. Untracked files travel as hunks rather than via `git add -N` because a capture must never rewrite the user's index, and the snapshot denylist filters the untracked list so a secret cannot leak through a hunk the archive would refuse. A clean worktree captures no patch and restores exactly as before, so the change is strictly additive.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>Dirty git repos restore to the exact uncommitted state instead of a mass re-overwrite. Adds an optional manifest field; manifests from older builds are unchanged. A patch that cannot apply (different base commit) is reported with the remedy, not silently dropped.</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>If restore ever needs to land local, uncommitted work on a checkout whose history diverged, the patch apply would need a 3-way merge strategy rather than the current apply-only.</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Assistant</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Decided</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>BUG-037</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>